<commit_message>
Rebuild for new 3-template English design (yellow/blue/red) + signature
- New artwork: three English templates (yellow, blue, red); Georgian removed.
  Templates 1 & 2 keep COURSE/LEVEL/PERIOD; template 3 (red) has COURSE/PERIOD only.
- Cambridge English Educational Partner badge is part of the artwork (baked in).
- Stamps app/signature.png (principal signature) above the PRINCIPAL label on
  every certificate; optional (skipped if the file is absent).
- Name in Red Hat Display Medium, values in Bold; layout recalibrated per variant.
- Drops Georgian fonts (BPG/LGV) and unused weights; updates UI, samples, tests, README.
</commit_message>
<xml_diff>
--- a/app/samples/certificate-template-1-sample.xlsx
+++ b/app/samples/certificate-template-1-sample.xlsx
@@ -429,10 +429,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ELIZAVETA</v>
+        <v>Elizaveta</v>
       </c>
       <c r="B2" t="str">
-        <v>DATUKISHVILI</v>
+        <v>Datukishvili</v>
       </c>
       <c r="C2" t="str">
         <v>General English</v>

</xml_diff>

<commit_message>
Rebuild for new design: Calibri fonts, Hours, certificate numbers + QR
- New 3-template artwork (yellow/blue = English, red = Art); adds an HOURS field
  and a single-line PERIOD; the principal signature is now baked into the template.
- Fonts: name = Red Hat Display Medium; values = Calibri Bold; certificate number
  = Calibri Light (font files uploaded to the repo).
- Generates the certificate number L<branch><subject>-<year>-<seq>:
  branch (Vake/Krtsanisi) + start number chosen in a new numbering step; subject
  from the template; year from the dates; sequence auto-increments.
- Renders a per-certificate QR code encoding https://levels.ge/verify/<number>
  (bundled qrcode-generator); verified it decodes correctly.
- Recalibrated all field positions/whiteouts to the new layout; updated UI,
  samples, tests and README.
</commit_message>
<xml_diff>
--- a/app/samples/certificate-template-1-sample.xlsx
+++ b/app/samples/certificate-template-1-sample.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -405,6 +405,7 @@
     <col min="4" max="4" width="24.83203125" customWidth="1"/>
     <col min="5" max="5" width="24.83203125" customWidth="1"/>
     <col min="6" max="6" width="24.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -421,9 +422,12 @@
         <v>Level</v>
       </c>
       <c r="E1" t="str">
+        <v>Hours</v>
+      </c>
+      <c r="F1" t="str">
         <v>Start Date</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>End Date</v>
       </c>
     </row>
@@ -441,9 +445,12 @@
         <v>Intermediate</v>
       </c>
       <c r="E2" t="str">
+        <v>48</v>
+      </c>
+      <c r="F2" t="str">
         <v>2026-01-16</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>2026-06-16</v>
       </c>
     </row>
@@ -460,16 +467,19 @@
       <c r="D3" t="str">
         <v>Beginner</v>
       </c>
-      <c r="E3" t="str">
+      <c r="E3">
+        <v>36</v>
+      </c>
+      <c r="F3" t="str">
         <v>2026-02-01</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>2026-07-01</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>